<commit_message>
update template excel file
</commit_message>
<xml_diff>
--- a/LAB4/Lab4_BVT.xlsx
+++ b/LAB4/Lab4_BVT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29E6032-A115-488C-86D0-038CFFDF0007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC6D60E-B3E4-406D-9C8B-170BD294AF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="71">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -238,6 +238,9 @@
   </si>
   <si>
     <t>17/7/2026</t>
+  </si>
+  <si>
+    <t>Out of range</t>
   </si>
 </sst>
 </file>
@@ -300,7 +303,6 @@
     </font>
     <font>
       <sz val="18"/>
-      <color rgb="FFFF0000"/>
       <name val="TH SarabunPSK"/>
       <family val="2"/>
     </font>
@@ -488,7 +490,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -522,6 +523,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -902,7 +904,9 @@
       <c r="C3" s="3">
         <v>13</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="17"/>
@@ -911,9 +915,15 @@
       <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="B4" s="6">
+        <v>19</v>
+      </c>
+      <c r="C4" s="6">
+        <v>17</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -932,8 +942,12 @@
         <v>40</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19"/>
+      <c r="C6" s="18">
+        <v>30</v>
+      </c>
+      <c r="D6" s="19">
+        <v>2</v>
+      </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="20"/>
@@ -961,15 +975,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="25"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1000,12 +1014,12 @@
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1029,12 +1043,12 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1058,10 +1072,10 @@
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1096,21 +1110,21 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="24.9" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="33" t="s">
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="33" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1127,7 +1141,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A8" s="33"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1137,9 +1151,9 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="34"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="33"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1169,8 +1183,12 @@
       <c r="E9" s="6">
         <v>8</v>
       </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="F9" s="6">
+        <v>8</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A10" s="6" t="s">
@@ -1188,8 +1206,12 @@
       <c r="E10" s="6">
         <v>8</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="F10" s="6">
+        <v>8</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A11" s="6" t="s">
@@ -1207,8 +1229,12 @@
       <c r="E11" s="6">
         <v>10</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="F11" s="6">
+        <v>10</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1230,8 +1256,12 @@
       <c r="E12" s="6">
         <v>11</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="F12" s="6">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1253,8 +1283,12 @@
       <c r="E13" s="6">
         <v>12</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="F13" s="6">
+        <v>12</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1276,8 +1310,12 @@
       <c r="E14" s="6">
         <v>12</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="F14" s="6">
+        <v>12</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1299,8 +1337,12 @@
       <c r="E15" s="6">
         <v>12</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="F15" s="6">
+        <v>12</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1322,8 +1364,12 @@
       <c r="E16" s="6">
         <v>8</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="F16" s="6">
+        <v>8</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1345,8 +1391,12 @@
       <c r="E17" s="6">
         <v>8</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="F17" s="6">
+        <v>8</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.7">
@@ -1365,8 +1415,12 @@
       <c r="E18" s="6">
         <v>9</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="F18" s="6">
+        <v>9</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1388,8 +1442,12 @@
       <c r="E19" s="6">
         <v>9</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="F19" s="6">
+        <v>9</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A20" s="6" t="s">
@@ -1407,8 +1465,12 @@
       <c r="E20" s="6">
         <v>11</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="F20" s="6">
+        <v>11</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A21" s="6" t="s">
@@ -1426,8 +1488,12 @@
       <c r="E21" s="6">
         <v>11</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="F21" s="6">
+        <v>11</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1506,15 +1572,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="25"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1531,20 +1597,26 @@
       <c r="J2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
+      <c r="K2" s="6">
+        <v>24</v>
+      </c>
+      <c r="L2" s="6">
+        <v>39</v>
+      </c>
+      <c r="M2" s="6">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
+      <c r="B3" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1554,20 +1626,26 @@
       <c r="J3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
+      <c r="K3" s="6">
+        <v>25</v>
+      </c>
+      <c r="L3" s="6">
+        <v>40</v>
+      </c>
+      <c r="M3" s="6">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1577,18 +1655,24 @@
       <c r="J4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
+      <c r="K4" s="6">
+        <v>26</v>
+      </c>
+      <c r="L4" s="6">
+        <v>41</v>
+      </c>
+      <c r="M4" s="6">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="28"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1598,45 +1682,63 @@
       <c r="J5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
+      <c r="K5" s="6">
+        <v>42</v>
+      </c>
+      <c r="L5" s="6">
+        <v>70</v>
+      </c>
+      <c r="M5" s="6">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.7">
       <c r="J6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
+      <c r="K6" s="6">
+        <v>60</v>
+      </c>
+      <c r="L6" s="6">
+        <v>219</v>
+      </c>
+      <c r="M6" s="6">
+        <v>29</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="24.9" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="33" t="s">
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="G7" s="33" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+      <c r="K7" s="6">
+        <v>61</v>
+      </c>
+      <c r="L7" s="6">
+        <v>220</v>
+      </c>
+      <c r="M7" s="6">
+        <v>30</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A8" s="33"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1646,48 +1748,90 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="34"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="33"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="K8" s="6">
+        <v>62</v>
+      </c>
+      <c r="L8" s="6">
+        <v>221</v>
+      </c>
+      <c r="M8" s="6">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="B9" s="6">
+        <v>24</v>
+      </c>
+      <c r="C9" s="6">
+        <v>70</v>
+      </c>
+      <c r="D9" s="6">
+        <v>20</v>
+      </c>
+      <c r="E9" s="34">
+        <v>7</v>
+      </c>
+      <c r="F9" s="6">
+        <v>7</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="B10" s="6">
+        <v>25</v>
+      </c>
+      <c r="C10" s="6">
+        <v>70</v>
+      </c>
+      <c r="D10" s="6">
+        <v>20</v>
+      </c>
+      <c r="E10" s="6">
+        <v>8</v>
+      </c>
+      <c r="F10" s="6">
+        <v>8</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="B11" s="6">
+        <v>26</v>
+      </c>
+      <c r="C11" s="6">
+        <v>70</v>
+      </c>
+      <c r="D11" s="6">
+        <v>20</v>
+      </c>
+      <c r="E11" s="6">
+        <v>8</v>
+      </c>
+      <c r="F11" s="6">
+        <v>8</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1697,12 +1841,24 @@
       <c r="A12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="B12" s="6">
+        <v>42</v>
+      </c>
+      <c r="C12" s="6">
+        <v>70</v>
+      </c>
+      <c r="D12" s="6">
+        <v>20</v>
+      </c>
+      <c r="E12" s="6">
+        <v>10</v>
+      </c>
+      <c r="F12" s="6">
+        <v>10</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1712,12 +1868,24 @@
       <c r="A13" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="B13" s="6">
+        <v>60</v>
+      </c>
+      <c r="C13" s="6">
+        <v>70</v>
+      </c>
+      <c r="D13" s="6">
+        <v>20</v>
+      </c>
+      <c r="E13" s="6">
+        <v>11</v>
+      </c>
+      <c r="F13" s="6">
+        <v>11</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1727,12 +1895,24 @@
       <c r="A14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="B14" s="6">
+        <v>61</v>
+      </c>
+      <c r="C14" s="6">
+        <v>70</v>
+      </c>
+      <c r="D14" s="6">
+        <v>20</v>
+      </c>
+      <c r="E14" s="6">
+        <v>12</v>
+      </c>
+      <c r="F14" s="6">
+        <v>12</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1742,12 +1922,24 @@
       <c r="A15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="B15" s="6">
+        <v>62</v>
+      </c>
+      <c r="C15" s="6">
+        <v>70</v>
+      </c>
+      <c r="D15" s="6">
+        <v>20</v>
+      </c>
+      <c r="E15" s="6">
+        <v>12</v>
+      </c>
+      <c r="F15" s="6">
+        <v>12</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1757,12 +1949,24 @@
       <c r="A16" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="B16" s="6">
+        <v>42</v>
+      </c>
+      <c r="C16" s="6">
+        <v>39</v>
+      </c>
+      <c r="D16" s="6">
+        <v>20</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1772,24 +1976,48 @@
       <c r="A17" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="B17" s="6">
+        <v>42</v>
+      </c>
+      <c r="C17" s="6">
+        <v>40</v>
+      </c>
+      <c r="D17" s="6">
+        <v>20</v>
+      </c>
+      <c r="E17" s="6">
+        <v>12</v>
+      </c>
+      <c r="F17" s="6">
+        <v>12</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="B18" s="6">
+        <v>42</v>
+      </c>
+      <c r="C18" s="6">
+        <v>41</v>
+      </c>
+      <c r="D18" s="6">
+        <v>20</v>
+      </c>
+      <c r="E18" s="6">
+        <v>12</v>
+      </c>
+      <c r="F18" s="6">
+        <v>12</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1799,34 +2027,70 @@
       <c r="A19" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="B19" s="6">
+        <v>42</v>
+      </c>
+      <c r="C19" s="6">
+        <v>219</v>
+      </c>
+      <c r="D19" s="6">
+        <v>20</v>
+      </c>
+      <c r="E19" s="6">
+        <v>8</v>
+      </c>
+      <c r="F19" s="6">
+        <v>8</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="B20" s="6">
+        <v>42</v>
+      </c>
+      <c r="C20" s="6">
+        <v>220</v>
+      </c>
+      <c r="D20" s="6">
+        <v>20</v>
+      </c>
+      <c r="E20" s="6">
+        <v>8</v>
+      </c>
+      <c r="F20" s="6">
+        <v>8</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.7">
       <c r="A21" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="B21" s="6">
+        <v>42</v>
+      </c>
+      <c r="C21" s="22">
+        <v>221</v>
+      </c>
+      <c r="D21" s="6">
+        <v>20</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1836,12 +2100,24 @@
       <c r="A22" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
+      <c r="B22" s="6">
+        <v>42</v>
+      </c>
+      <c r="C22" s="6">
+        <v>70</v>
+      </c>
+      <c r="D22" s="6">
+        <v>11</v>
+      </c>
+      <c r="E22" s="6">
+        <v>7</v>
+      </c>
+      <c r="F22" s="6">
+        <v>7</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -1851,12 +2127,24 @@
       <c r="A23" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+      <c r="B23" s="6">
+        <v>42</v>
+      </c>
+      <c r="C23" s="6">
+        <v>70</v>
+      </c>
+      <c r="D23" s="6">
+        <v>12</v>
+      </c>
+      <c r="E23" s="6">
+        <v>9</v>
+      </c>
+      <c r="F23" s="6">
+        <v>9</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -1866,12 +2154,24 @@
       <c r="A24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+      <c r="B24" s="6">
+        <v>42</v>
+      </c>
+      <c r="C24" s="6">
+        <v>70</v>
+      </c>
+      <c r="D24" s="6">
+        <v>13</v>
+      </c>
+      <c r="E24" s="6">
+        <v>9</v>
+      </c>
+      <c r="F24" s="6">
+        <v>9</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -1881,12 +2181,24 @@
       <c r="A25" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+      <c r="B25" s="6">
+        <v>42</v>
+      </c>
+      <c r="C25" s="6">
+        <v>70</v>
+      </c>
+      <c r="D25" s="6">
+        <v>29</v>
+      </c>
+      <c r="E25" s="6">
+        <v>11</v>
+      </c>
+      <c r="F25" s="6">
+        <v>11</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -1896,12 +2208,24 @@
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
+      <c r="B26" s="6">
+        <v>42</v>
+      </c>
+      <c r="C26" s="6">
+        <v>70</v>
+      </c>
+      <c r="D26" s="6">
+        <v>30</v>
+      </c>
+      <c r="E26" s="6">
+        <v>11</v>
+      </c>
+      <c r="F26" s="6">
+        <v>11</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -1911,12 +2235,24 @@
       <c r="A27" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
+      <c r="B27" s="6">
+        <v>42</v>
+      </c>
+      <c r="C27" s="6">
+        <v>70</v>
+      </c>
+      <c r="D27" s="6">
+        <v>31</v>
+      </c>
+      <c r="E27" s="6">
+        <v>11</v>
+      </c>
+      <c r="F27" s="6">
+        <v>11</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.7">

</xml_diff>

<commit_message>
update environment in template excel file
</commit_message>
<xml_diff>
--- a/LAB4/Lab4_BVT.xlsx
+++ b/LAB4/Lab4_BVT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sqa-2026-lab\SQA\LAB4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC6D60E-B3E4-406D-9C8B-170BD294AF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF4585A-1BB0-4BD3-A607-0EB0A50E86C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="71">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -234,13 +234,13 @@
     <t>หทัยพัทธ วิสุทธิธรรม</t>
   </si>
   <si>
-    <t>14/7/2026</t>
-  </si>
-  <si>
     <t>17/7/2026</t>
   </si>
   <si>
     <t>Out of range</t>
+  </si>
+  <si>
+    <t>Window 11, JUnit6, specs Intel Core i512450H RAM 16 GB DDR4</t>
   </si>
 </sst>
 </file>
@@ -490,6 +490,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -499,6 +500,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -508,22 +515,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -975,15 +975,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="26"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1014,12 +1014,12 @@
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1043,12 +1043,12 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1072,15 +1072,17 @@
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="28"/>
+      <c r="B5" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>8</v>
@@ -1113,18 +1115,18 @@
       <c r="A7" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="32" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="34" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1153,7 +1155,7 @@
       </c>
       <c r="E8" s="32"/>
       <c r="F8" s="32"/>
-      <c r="G8" s="33"/>
+      <c r="G8" s="34"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1572,15 +1574,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.7">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="26"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1611,12 +1613,12 @@
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
+      <c r="B3" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1640,12 +1642,12 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1669,10 +1671,12 @@
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="28"/>
+      <c r="B5" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1710,18 +1714,18 @@
       <c r="A7" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
       <c r="E7" s="32" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="34" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1750,7 +1754,7 @@
       </c>
       <c r="E8" s="32"/>
       <c r="F8" s="32"/>
-      <c r="G8" s="33"/>
+      <c r="G8" s="34"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1777,7 +1781,7 @@
       <c r="D9" s="6">
         <v>20</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="23">
         <v>7</v>
       </c>
       <c r="F9" s="6">
@@ -1959,10 +1963,10 @@
         <v>20</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>36</v>
@@ -2083,10 +2087,10 @@
         <v>20</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>36</v>

</xml_diff>